<commit_message>
vault backup: 2026-10-08 11:34:09
</commit_message>
<xml_diff>
--- a/WebLogic-VN-confirmed.xlsx
+++ b/WebLogic-VN-confirmed.xlsx
@@ -486,122 +486,122 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>https://congbothongtin.ssc.gov.vn</t>
+          <t>http://agimexpharm.com:8081</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>103.3.252.107</t>
+          <t>113.161.212.113:8081</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Long Xuyen</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>https://congbothongtin.ssc.gov.vn:7002</t>
+          <t>http://dlp.com.tw:7001</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>103.3.252.107:7002</t>
+          <t>113.160.129.228:7001</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>https://dvctn.vst.mof.gov.vn</t>
+          <t>http://dlp.com.tw:8888</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>45.120.230.41</t>
+          <t>113.160.129.148:8888</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>https://epayment.customs.gov.vn</t>
+          <t>http://dlp.com.tw:8888</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>103.248.160.36</t>
+          <t>113.160.129.155:8888</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Customs Statistics</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>https://ids.ssc.gov.vn</t>
+          <t>http://dlp.com.tw:8888</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>103.3.252.106</t>
+          <t>113.160.129.228:8888</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>https://ids.ssc.gov.vn:7002</t>
+          <t>http://dlp.com.tw:8888</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>103.3.252.106:7002</t>
+          <t>123.25.63.26:8888</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -611,542 +611,662 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>https://sso.vietinbank.vn</t>
+          <t>http://quickconnect.to:82</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
+          <t>14.241.227.70:82</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>http://sso.vietinbank.vn</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
           <t>203.189.29.33</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>VIETNAM Joint Stock Commercial Bank for Industry and Trade</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>http://103.104.121.206:9999</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>103.104.121.206:9999</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>http://xboss.vn:9999</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>103.104.121.208:9999</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>http://103.104.121.207:9999</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>103.104.121.207:9999</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>https://congbothongtin.ssc.gov.vn</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>103.3.252.107</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>https://dailybanxetai.com</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>123.30.208.19</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>https://dailybanxetai.com:8098</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>123.30.208.19:8098</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>https://dvctn.vst.mof.gov.vn</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>45.120.230.41</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>https://epayment.customs.gov.vn</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>103.248.160.36</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Department of Information Technology and Customs Statistics</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>https://ids.ssc.gov.vn</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>103.3.252.106</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>https://kimdental.vn</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>42.115.41.28</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>https://mfmldb.com.vn:8184</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>14.238.93.114:8184</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Viet Storage Technology Joint Stock Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>http://103.104.121.208:9999</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>103.104.121.208:9999</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>https://mfmldb.com.vn:8185</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>14.238.93.114:8185</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Viet Storage Technology Joint Stock Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>http://103.82.192.168</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>103.82.192.168</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>http://113.160.129.148:8888</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>113.160.129.148:8888</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>Hai Duong</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>https://mof.gov.vn</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>45.120.230.40</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>https://mof.gov.vn</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>45.120.230.51</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>https://mps.gov.vn</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>42.1.75.65</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Mobifone Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>https://pritos.cloud:3068</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>115.75.20.142:3068</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Thi Tran Long Dien</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Viettel Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>https://pvfcco.com.vn</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>14.238.99.83</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Tan An</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>http://113.160.129.149:8888</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>113.160.129.149:8888</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
-        <is>
-          <t>Hai Duong</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>https://pvfcco.com.vn</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>14.238.99.84</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Tan An</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>http://113.160.129.155:8888</t>
-        </is>
-      </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>113.160.129.155:8888</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>Hai Duong</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>https://temxacthuc.vn:8081</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>123.30.208.19:8081</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>http://113.160.129.228:7001</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>113.160.129.228:7001</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>Hai Duong</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>https://thongbaotenmien.vn</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>203.119.73.12</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam Internet network information center (VNNIC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>https://toaan.gov.vn</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>123.30.24.180</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>http://113.160.129.228:8888</t>
-        </is>
-      </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>113.160.129.228:8888</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>Hai Duong</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>http://113.160.201.159:7001</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>113.160.201.159:7001</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>http://113.161.212.113:8081</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>113.161.212.113:8081</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Long Xuyen</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>http://113.161.43.248:9001</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>113.161.43.248:9001</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>http://113.163.187.3:27001</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>113.163.187.3:27001</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>http://113.185.19.167:8080</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>113.185.19.167:8080</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>http://115.75.20.142:3068</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>115.75.20.142:3068</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>http://117.4.241.247:1112</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>117.4.241.247:1112</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr"/>
-      <c r="D24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>http://117.4.32.40:1111</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>117.4.32.40:1111</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr"/>
-      <c r="D25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>http://118.69.182.224:8879</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>118.69.182.224:8879</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr"/>
-      <c r="D26" s="3" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>http://118.69.32.193:3068</t>
-        </is>
-      </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>118.69.32.193:3068</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr"/>
-      <c r="D27" s="3" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>http://123.25.63.26:8888</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>123.25.63.26:8888</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr"/>
-      <c r="D28" s="3" t="inlineStr"/>
-    </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>http://123.25.63.30:8888</t>
-        </is>
-      </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>123.25.63.30:8888</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr"/>
-      <c r="D29" s="3" t="inlineStr"/>
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>https://vinpro.net</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>103.238.209.204</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
+        </is>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
-        <is>
-          <t>http://123.31.31.119:49163</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>123.31.31.119:49163</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>https://xsmb360.com</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>103.82.194.3</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Tra Vinh</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>CLOUDFLY CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>http://123.31.31.125:49163</t>
+          <t>http://103.104.121.206:9999</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>123.31.31.125:49163</t>
+          <t>103.104.121.206:9999</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>http://123.31.36.63:8002</t>
+          <t>http://103.104.121.207:9999</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>123.31.36.63:8002</t>
+          <t>103.104.121.207:9999</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>http://14.238.93.114:8184</t>
+          <t>http://113.160.129.149:8888</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>14.238.93.114:8184</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr"/>
+          <t>113.160.129.149:8888</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Hai Duong</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>http://14.238.93.114:8185</t>
+          <t>http://113.160.201.159:7001</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>14.238.93.114:8185</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr"/>
-      <c r="D34" s="3" t="inlineStr"/>
+          <t>113.160.201.159:7001</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Thai Binh</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>http://14.238.93.114:9184</t>
+          <t>http://113.161.43.248:9001</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>14.238.93.114:9184</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr"/>
+          <t>113.161.43.248:9001</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>http://14.238.93.114:9185</t>
+          <t>http://113.163.187.3:27001</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>14.238.93.114:9185</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr"/>
-      <c r="D36" s="3" t="inlineStr"/>
+          <t>113.163.187.3:27001</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Phan Rang-Thap Cham</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>http://14.241.227.70:82</t>
+          <t>http://113.185.0.60:8080</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>14.241.227.70:82</t>
+          <t>113.185.0.60:8080</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -1158,17 +1278,17 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>http://14.241.253.96:8081</t>
+          <t>http://113.185.19.167:8080</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>14.241.253.96:8081</t>
+          <t>113.185.19.167:8080</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -1180,132 +1300,144 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>http://14.241.253.96:8082</t>
+          <t>http://117.4.241.247:1112</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>14.241.253.96:8082</t>
+          <t>117.4.241.247:1112</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>http://160.191.101.129:9001</t>
+          <t>http://117.4.32.40:1111</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>160.191.101.129:9001</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr"/>
+          <t>117.4.32.40:1111</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Gplay Joint Stock Company</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>http://171.244.38.92:7001</t>
+          <t>http://118.69.182.224:8879</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>171.244.38.92:7001</t>
+          <t>118.69.182.224:8879</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Bien Hoa</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>http://183.91.187.108:8888</t>
+          <t>http://123.25.63.30:8888</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>183.91.187.108:8888</t>
+          <t>123.25.63.30:8888</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>http://183.91.187.108:8890</t>
+          <t>http://123.31.31.119:49163</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>183.91.187.108:8890</t>
+          <t>123.31.31.119:49163</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>http://203.119.73.12</t>
+          <t>http://123.31.31.125:49163</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>203.119.73.12</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr"/>
-      <c r="D44" s="3" t="inlineStr"/>
+          <t>123.31.31.125:49163</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>http://210.211.98.79:8080</t>
+          <t>http://123.31.36.63:8002</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>210.211.98.79:8080</t>
+          <t>123.31.36.63:8002</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -1315,119 +1447,151 @@
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>Viettel - CHT Company Ltd</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>http://210.211.98.79:8081</t>
+          <t>http://14.241.253.96:8081</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>210.211.98.79:8081</t>
+          <t>14.241.253.96:8081</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>Viettel - CHT Company Ltd</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>http://210.211.99.108:8080</t>
+          <t>http://14.241.253.96:8082</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>210.211.99.108:8080</t>
+          <t>14.241.253.96:8082</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Viettel - CHT Company Ltd</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>http://42.115.41.28</t>
+          <t>http://160.191.101.129:9001</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>42.115.41.28</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr"/>
-      <c r="D48" s="3" t="inlineStr"/>
+          <t>160.191.101.129:9001</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Gplay Joint Stock Company</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>http://42.116.12.202:9001</t>
+          <t>http://171.244.38.92:7001</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>42.116.12.202:9001</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr"/>
-      <c r="D49" s="3" t="inlineStr"/>
+          <t>171.244.38.92:7001</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Viettel Group</t>
+        </is>
+      </c>
     </row>
     <row r="50">
-      <c r="A50" s="3" t="inlineStr">
-        <is>
-          <t>http://42.118.60.193:7001</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>42.118.60.193:7001</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr"/>
-      <c r="D50" s="3" t="inlineStr"/>
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>http://183.91.187.108:8888</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>183.91.187.108:8888</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>http://49.213.88.170:7001</t>
+          <t>http://210.211.98.79:8080</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>49.213.88.170:7001</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr"/>
-      <c r="D51" s="3" t="inlineStr"/>
+          <t>210.211.98.79:8080</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Viettel - CHT Company Ltd</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>https://103.238.209.174</t>
+          <t>http://210.211.98.79:8081</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>103.238.209.174</t>
+          <t>210.211.98.79:8081</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -1437,63 +1601,63 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="3" t="inlineStr">
-        <is>
-          <t>https://103.238.209.204</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>103.238.209.204</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>http://210.211.99.108:8080</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>210.211.99.108:8080</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>https://103.82.194.3</t>
+          <t>http://42.116.12.202:9001</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>103.82.194.3</t>
+          <t>42.116.12.202:9001</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Tra Vinh</t>
+          <t>Thu Dau Mot</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>CLOUDFLY CORPORATION</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>https://113.185.0.60:8080</t>
+          <t>http://42.118.60.193:7001</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>113.185.0.60:8080</t>
+          <t>42.118.60.193:7001</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -1503,41 +1667,41 @@
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>https://123.30.208.19</t>
+          <t>http://49.213.88.170:7001</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19</t>
+          <t>49.213.88.170:7001</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>VNG Corporation</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>https://123.30.208.19:8081</t>
+          <t>https://103.238.209.174</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19:8081</t>
+          <t>103.238.209.174</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -1547,112 +1711,112 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="3" t="inlineStr">
-        <is>
-          <t>https://123.30.208.19:8098</t>
-        </is>
-      </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>123.30.208.19:8098</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>https://103.3.252.106:7002</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>103.3.252.106:7002</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
-        <is>
-          <t>https://123.30.24.180</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>123.30.24.180</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>https://103.3.252.107:7002</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>103.3.252.107:7002</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>https://123.31.36.60</t>
+          <t>https://103.82.192.168</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>123.31.36.60</t>
+          <t>103.82.192.168</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Da Nang</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>CLOUDFLY CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="3" t="inlineStr">
-        <is>
-          <t>https://14.238.99.83</t>
-        </is>
-      </c>
-      <c r="B61" s="3" t="inlineStr">
-        <is>
-          <t>14.238.99.83</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr">
-        <is>
-          <t>Tan An</t>
-        </is>
-      </c>
-      <c r="D61" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>https://118.69.32.193:3068</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>118.69.32.193:3068</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Thu Dau Mot</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>https://14.238.99.84</t>
+          <t>https://123.31.36.60</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>14.238.99.84</t>
+          <t>123.31.36.60</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Tan An</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -1662,134 +1826,134 @@
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="3" t="inlineStr">
-        <is>
-          <t>https://14.248.84.7</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>14.248.84.7</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D63" s="3" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>https://14.238.93.114:9184</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>14.238.93.114:9184</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="3" t="inlineStr">
-        <is>
-          <t>https://210.211.99.108</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>210.211.99.108</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Viettel - CHT Company Ltd</t>
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>https://14.238.93.114:9185</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>14.238.93.114:9185</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>https://210.245.45.90</t>
+          <t>https://14.248.84.7</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>210.245.45.90</t>
+          <t>14.248.84.7</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>https://183.91.187.108:8890</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>183.91.187.108:8890</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>Dai IP cap cho Cong ty TNHH Nguon Viet Nam</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="3" t="inlineStr">
-        <is>
-          <t>https://42.1.75.65</t>
-        </is>
-      </c>
-      <c r="B66" s="3" t="inlineStr">
-        <is>
-          <t>42.1.75.65</t>
-        </is>
-      </c>
-      <c r="C66" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D66" s="3" t="inlineStr">
-        <is>
-          <t>Mobifone Corporation</t>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="3" t="inlineStr">
-        <is>
-          <t>https://45.120.230.40</t>
-        </is>
-      </c>
-      <c r="B67" s="3" t="inlineStr">
-        <is>
-          <t>45.120.230.40</t>
-        </is>
-      </c>
-      <c r="C67" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="D67" s="3" t="inlineStr">
-        <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>https://210.211.99.108</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>210.211.99.108</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>https://45.120.230.51</t>
+          <t>https://210.245.45.90</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.51</t>
+          <t>210.245.45.90</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Dai IP cap cho Cong ty TNHH Nguon Viet Nam</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-10-08 11:49:19
</commit_message>
<xml_diff>
--- a/WebLogic-VN-confirmed.xlsx
+++ b/WebLogic-VN-confirmed.xlsx
@@ -10,7 +10,7 @@
     <sheet name="WebLogic VN" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WebLogic VN'!$A$1:$D$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WebLogic VN'!$A$1:$E$68</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -452,13 +452,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D68"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,10 +475,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Thành phố</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Tổ chức</t>
         </is>
@@ -486,20 +492,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>http://agimexpharm.com:8081</t>
+          <t>http://apv1.dlp.com.tw:8888</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>113.161.212.113:8081</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Long Xuyen</t>
-        </is>
-      </c>
+          <t>113.160.129.148:8888</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Hai Duong</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -508,73 +515,80 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>http://dlp.com.tw:7001</t>
+          <t>http://apvn2.dlp.com.tw:8888</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>113.160.129.228:7001</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
+          <t>113.160.129.155:8888</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>http://dlp.com.tw:8888</t>
+          <t>http://apvn3.dlp.com.tw:8888</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>113.160.129.148:8888</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Hai Duong</t>
-        </is>
-      </c>
+          <t>123.25.63.26:8888</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>http://dlp.com.tw:8888</t>
+          <t>http://apvs1.dlp.com.tw:7001</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>113.160.129.155:8888</t>
+          <t>113.160.129.228:7001</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>http://dlp.com.tw:8888</t>
+          <t>http://apvs1.dlp.com.tw:8888</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -582,12 +596,13 @@
           <t>113.160.129.228:8888</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -596,42 +611,44 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>http://dlp.com.tw:8888</t>
+          <t>http://gasdaiminhquang.direct.quickconnect.to:82</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>123.25.63.26:8888</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>14.241.227.70:82</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>http://quickconnect.to:82</t>
+          <t>http://hddt.agimexpharm.com:8081</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>14.241.227.70:82</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
+          <t>113.161.212.113:8081</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Long Xuyen</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -640,44 +657,46 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>http://sso.vietinbank.vn</t>
+          <t>http://mail.xboss.vn:9999</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>203.189.29.33</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>103.104.121.208:9999</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>VIETNAM Joint Stock Commercial Bank for Industry and Trade</t>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>http://xboss.vn:9999</t>
+          <t>http://sso.vietinbank.vn</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>103.104.121.208:9999</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
+          <t>203.189.29.33</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Viet Storage Technology Joint Stock Company</t>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>VIETNAM Joint Stock Commercial Bank for Industry and Trade</t>
         </is>
       </c>
     </row>
@@ -692,12 +711,13 @@
           <t>103.3.252.107</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
@@ -706,7 +726,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>https://dailybanxetai.com</t>
+          <t>https://cskh.temxacthuc.vn</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -714,12 +734,13 @@
           <t>123.30.208.19</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -728,20 +749,21 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>https://dailybanxetai.com:8098</t>
+          <t>https://cskh.temxacthuc.vn:8081</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>123.30.208.19:8098</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>123.30.208.19:8081</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -758,12 +780,13 @@
           <t>45.120.230.41</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
@@ -780,12 +803,13 @@
           <t>103.248.160.36</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>Department of Information Technology and Customs Statistics</t>
         </is>
@@ -794,110 +818,119 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>https://ids.ssc.gov.vn</t>
+          <t>https://hrs.mfmldb.com.vn:8184</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>103.3.252.106</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>14.238.93.114:8184</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>https://kimdental.vn</t>
+          <t>https://hrs.mfmldb.com.vn:8185</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>42.115.41.28</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>14.238.93.114:8185</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>https://mfmldb.com.vn:8184</t>
+          <t>https://ids.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>14.238.93.114:8184</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
+          <t>103.3.252.106</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>https://mfmldb.com.vn:8185</t>
+          <t>https://kimdental.vn</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>14.238.93.114:8185</t>
+          <t>42.115.41.28</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>12.2.1.3.0</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.vn</t>
+          <t>https://mail.dailybanxetai.com:8098</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>45.120.230.40</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>123.30.208.19:8098</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
@@ -909,15 +942,16 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>45.120.230.51</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>45.120.230.40</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
@@ -926,66 +960,69 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>https://mps.gov.vn</t>
+          <t>https://mof.gov.vn</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>42.1.75.65</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>45.120.230.51</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Mobifone Corporation</t>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>https://pritos.cloud:3068</t>
+          <t>https://mps.gov.vn</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>115.75.20.142:3068</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>Thi Tran Long Dien</t>
-        </is>
-      </c>
+          <t>42.1.75.65</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Mobifone Corporation</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>https://pvfcco.com.vn</t>
+          <t>https://pritos.cloud:3068</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>14.238.99.83</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Tan An</t>
-        </is>
-      </c>
+          <t>115.75.20.142:3068</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Thi Tran Long Dien</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
@@ -997,15 +1034,16 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>14.238.99.84</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
+          <t>14.238.99.83</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Tan An</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1014,20 +1052,21 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>https://temxacthuc.vn:8081</t>
+          <t>https://pvfcco.com.vn</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>123.30.208.19:8081</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+          <t>14.238.99.84</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr"/>
       <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Tan An</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1044,12 +1083,13 @@
           <t>203.119.73.12</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="E27" s="2" t="inlineStr">
         <is>
           <t>Vietnam Internet network information center (VNNIC)</t>
         </is>
@@ -1066,12 +1106,13 @@
           <t>123.30.24.180</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C28" s="2" t="inlineStr"/>
       <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1088,12 +1129,13 @@
           <t>103.238.209.204</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C29" s="2" t="inlineStr"/>
       <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
@@ -1112,10 +1154,15 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
           <t>Tra Vinh</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>CLOUDFLY CORPORATION</t>
         </is>
@@ -1132,12 +1179,13 @@
           <t>103.104.121.206:9999</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="E31" s="3" t="inlineStr">
         <is>
           <t>Viet Storage Technology Joint Stock Company</t>
         </is>
@@ -1154,12 +1202,13 @@
           <t>103.104.121.207:9999</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>Viet Storage Technology Joint Stock Company</t>
         </is>
@@ -1176,12 +1225,13 @@
           <t>113.160.129.149:8888</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
         <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="E33" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1200,10 +1250,15 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
           <t>Thai Binh</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -1220,12 +1275,13 @@
           <t>113.161.43.248:9001</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="E35" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -1244,10 +1300,15 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
           <t>Phan Rang-Thap Cham</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -1264,12 +1325,13 @@
           <t>113.185.0.60:8080</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C37" s="3" t="inlineStr"/>
       <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1286,12 +1348,13 @@
           <t>113.185.19.167:8080</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C38" s="3" t="inlineStr"/>
       <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1310,10 +1373,15 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>10.3.6.0</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
         <is>
           <t>Viettel Group</t>
         </is>
@@ -1332,10 +1400,15 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>10.3.6.0</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>Viettel Group</t>
         </is>
@@ -1352,12 +1425,13 @@
           <t>118.69.182.224:8879</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="C41" s="3" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr">
         <is>
           <t>Bien Hoa</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="E41" s="3" t="inlineStr">
         <is>
           <t>FPT Telecom Company</t>
         </is>
@@ -1374,12 +1448,13 @@
           <t>123.25.63.30:8888</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C42" s="3" t="inlineStr"/>
       <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -1398,10 +1473,15 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>14.1.1.0.0</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
         <is>
           <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
@@ -1420,10 +1500,15 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>14.1.1.0.0</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
         <is>
           <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
@@ -1442,10 +1527,15 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>14.1.1.0.0</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1462,12 +1552,13 @@
           <t>14.241.253.96:8081</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C46" s="3" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="E46" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1484,12 +1575,13 @@
           <t>14.241.253.96:8082</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1506,12 +1598,13 @@
           <t>160.191.101.129:9001</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C48" s="3" t="inlineStr"/>
       <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
         <is>
           <t>Gplay Joint Stock Company</t>
         </is>
@@ -1530,10 +1623,15 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="E49" s="3" t="inlineStr">
         <is>
           <t>Viettel Group</t>
         </is>
@@ -1550,12 +1648,13 @@
           <t>183.91.187.108:8888</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
         </is>
@@ -1574,10 +1673,15 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>14.1.1.0.0</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
         <is>
           <t>Viettel - CHT Company Ltd</t>
         </is>
@@ -1596,10 +1700,15 @@
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>14.1.1.0.0</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
         <is>
           <t>Viettel - CHT Company Ltd</t>
         </is>
@@ -1618,10 +1727,15 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>14.1.1.0.0</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>Viettel - CHT Company Ltd</t>
         </is>
@@ -1638,12 +1752,13 @@
           <t>42.116.12.202:9001</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>Thu Dau Mot</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>FPT Telecom Company</t>
         </is>
@@ -1662,10 +1777,15 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>10.3.6.0</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
         <is>
           <t>FPT Telecom Company</t>
         </is>
@@ -1684,10 +1804,15 @@
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>VNG Corporation</t>
         </is>
@@ -1704,12 +1829,13 @@
           <t>103.238.209.174</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C57" s="3" t="inlineStr"/>
       <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
         <is>
           <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
@@ -1726,12 +1852,13 @@
           <t>103.3.252.106:7002</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C58" s="2" t="inlineStr"/>
       <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
@@ -1748,12 +1875,13 @@
           <t>103.3.252.107:7002</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C59" s="2" t="inlineStr"/>
       <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
         <is>
           <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
@@ -1772,10 +1900,15 @@
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
           <t>Da Nang</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="E60" s="3" t="inlineStr">
         <is>
           <t>CLOUDFLY CORPORATION</t>
         </is>
@@ -1792,12 +1925,13 @@
           <t>118.69.32.193:3068</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr">
+      <c r="C61" s="2" t="inlineStr"/>
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>Thu Dau Mot</t>
         </is>
       </c>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="E61" s="2" t="inlineStr">
         <is>
           <t>FPT Telecom Company</t>
         </is>
@@ -1814,12 +1948,13 @@
           <t>123.31.36.60</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C62" s="3" t="inlineStr"/>
       <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1836,12 +1971,13 @@
           <t>14.238.93.114:9184</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr"/>
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="E63" s="2" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -1858,12 +1994,13 @@
           <t>14.238.93.114:9185</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr"/>
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="E64" s="2" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -1880,12 +2017,13 @@
           <t>14.248.84.7</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C65" s="3" t="inlineStr"/>
       <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1902,12 +2040,13 @@
           <t>183.91.187.108:8890</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="E66" s="2" t="inlineStr">
         <is>
           <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
         </is>
@@ -1924,12 +2063,13 @@
           <t>210.211.99.108</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
+      <c r="C67" s="2" t="inlineStr"/>
       <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
         <is>
           <t>Viettel - CHT Company Ltd</t>
         </is>
@@ -1946,19 +2086,20 @@
           <t>210.245.45.90</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr"/>
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr">
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>Dai IP cap cho Cong ty TNHH Nguon Viet Nam</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D68"/>
+  <autoFilter ref="A1:E68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-08 14:50:35
</commit_message>
<xml_diff>
--- a/WebLogic-VN-confirmed.xlsx
+++ b/WebLogic-VN-confirmed.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +30,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="4">
@@ -76,12 +80,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -495,18 +505,18 @@
           <t>http://apv1.dlp.com.tw:8888</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>113.160.129.148:8888</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -518,18 +528,18 @@
           <t>http://apvn2.dlp.com.tw:8888</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>113.160.129.155:8888</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -541,18 +551,18 @@
           <t>http://apvn3.dlp.com.tw:8888</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>123.25.63.26:8888</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -564,22 +574,22 @@
           <t>http://apvs1.dlp.com.tw:7001</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>113.160.129.228:7001</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -591,18 +601,18 @@
           <t>http://apvs1.dlp.com.tw:8888</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>113.160.129.228:8888</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -614,18 +624,18 @@
           <t>http://gasdaiminhquang.direct.quickconnect.to:82</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>14.241.227.70:82</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -637,18 +647,18 @@
           <t>http://hddt.agimexpharm.com:8081</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>113.161.212.113:8081</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Long Xuyen</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -660,18 +670,18 @@
           <t>http://mail.xboss.vn:9999</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>103.104.121.208:9999</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr"/>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Viet Storage Technology Joint Stock Company</t>
         </is>
@@ -683,18 +693,18 @@
           <t>http://sso.vietinbank.vn</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>203.189.29.33</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>VIETNAM Joint Stock Commercial Bank for Industry and Trade</t>
         </is>
@@ -706,18 +716,18 @@
           <t>https://congbothongtin.ssc.gov.vn</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>103.3.252.107</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
@@ -726,21 +736,21 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>https://cskh.temxacthuc.vn</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>123.30.208.19</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr"/>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+          <t>https://cskh.temxacthuc.vn:8081</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>123.30.208.19:8081</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -749,90 +759,90 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>https://cskh.temxacthuc.vn:8081</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>123.30.208.19:8081</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr"/>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>https://dvctn.vst.mof.gov.vn</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>45.120.230.41</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>https://dvctn.vst.mof.gov.vn</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>45.120.230.41</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr"/>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>https://epayment.customs.gov.vn</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>103.248.160.36</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Department of Information Technology and Customs Statistics</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>https://epayment.customs.gov.vn</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>103.248.160.36</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr"/>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Department of Information Technology and Customs Statistics</t>
+          <t>https://hrs.mfmldb.com.vn:8184</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>14.238.93.114:8184</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>https://hrs.mfmldb.com.vn:8184</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>14.238.93.114:8184</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr"/>
-      <c r="D16" s="2" t="inlineStr">
+          <t>https://hrs.mfmldb.com.vn:8185</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>14.238.93.114:8185</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -841,73 +851,73 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>https://hrs.mfmldb.com.vn:8185</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>14.238.93.114:8185</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr"/>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
+          <t>https://ids.ssc.gov.vn</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>103.3.252.106</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>https://ids.ssc.gov.vn</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>103.3.252.106</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr"/>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>https://kimdental.vn</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>42.115.41.28</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>12.2.1.3.0</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>https://kimdental.vn</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>42.115.41.28</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>12.2.1.3.0</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>FPT Telecom Company</t>
+          <t>https://mail.dailybanxetai.com</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>123.30.208.19</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
@@ -917,18 +927,18 @@
           <t>https://mail.dailybanxetai.com:8098</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>123.30.208.19:8098</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr"/>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -940,18 +950,18 @@
           <t>https://mof.gov.vn</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>45.120.230.40</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr"/>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
@@ -963,18 +973,18 @@
           <t>https://mof.gov.vn</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>45.120.230.51</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
@@ -986,18 +996,18 @@
           <t>https://mps.gov.vn</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>42.1.75.65</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
         <is>
           <t>Mobifone Corporation</t>
         </is>
@@ -1009,18 +1019,18 @@
           <t>https://pritos.cloud:3068</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>115.75.20.142:3068</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr">
         <is>
           <t>Thi Tran Long Dien</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Viettel Group</t>
         </is>
@@ -1032,18 +1042,18 @@
           <t>https://pvfcco.com.vn</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>14.238.99.83</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
         <is>
           <t>Tan An</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1055,18 +1065,18 @@
           <t>https://pvfcco.com.vn</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>14.238.99.84</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>Tan An</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1078,18 +1088,18 @@
           <t>https://thongbaotenmien.vn</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>203.119.73.12</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="3" t="inlineStr">
         <is>
           <t>Vietnam Internet network information center (VNNIC)</t>
         </is>
@@ -1101,18 +1111,18 @@
           <t>https://toaan.gov.vn</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>123.30.24.180</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1124,18 +1134,18 @@
           <t>https://vinpro.net</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>103.238.209.204</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
         <is>
           <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
@@ -1147,491 +1157,491 @@
           <t>https://xsmb360.com</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>103.82.194.3</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>Tra Vinh</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="3" t="inlineStr">
         <is>
           <t>CLOUDFLY CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>http://103.104.121.206:9999</t>
         </is>
       </c>
-      <c r="B31" s="3" t="inlineStr">
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>103.104.121.206:9999</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr"/>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E31" s="3" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+      <c r="A32" s="4" t="inlineStr">
         <is>
           <t>http://103.104.121.207:9999</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>103.104.121.207:9999</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr"/>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="5" t="inlineStr">
         <is>
           <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>http://113.160.129.149:8888</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>113.160.129.149:8888</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr"/>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Hai Duong</t>
         </is>
       </c>
-      <c r="E33" s="3" t="inlineStr">
+      <c r="E33" s="5" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+      <c r="A34" s="4" t="inlineStr">
         <is>
           <t>http://113.160.201.159:7001</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>113.160.201.159:7001</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>Thai Binh</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" s="5" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>http://113.161.43.248:9001</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
         <is>
           <t>113.161.43.248:9001</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr"/>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
+      <c r="E35" s="5" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>http://113.163.187.3:27001</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>113.163.187.3:27001</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>Phan Rang-Thap Cham</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" s="5" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="4" t="inlineStr">
         <is>
           <t>http://113.185.0.60:8080</t>
         </is>
       </c>
-      <c r="B37" s="3" t="inlineStr">
+      <c r="B37" s="5" t="inlineStr">
         <is>
           <t>113.185.0.60:8080</t>
         </is>
       </c>
-      <c r="C37" s="3" t="inlineStr"/>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr"/>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+      <c r="A38" s="4" t="inlineStr">
         <is>
           <t>http://113.185.19.167:8080</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B38" s="5" t="inlineStr">
         <is>
           <t>113.185.19.167:8080</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr"/>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="C38" s="5" t="inlineStr"/>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="4" t="inlineStr">
         <is>
           <t>http://117.4.241.247:1112</t>
         </is>
       </c>
-      <c r="B39" s="3" t="inlineStr">
+      <c r="B39" s="5" t="inlineStr">
         <is>
           <t>117.4.241.247:1112</t>
         </is>
       </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="C39" s="5" t="inlineStr">
         <is>
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
         <is>
           <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>http://117.4.32.40:1111</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
+      <c r="B40" s="5" t="inlineStr">
         <is>
           <t>117.4.32.40:1111</t>
         </is>
       </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C40" s="5" t="inlineStr">
         <is>
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
         <is>
           <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A41" s="4" t="inlineStr">
         <is>
           <t>http://118.69.182.224:8879</t>
         </is>
       </c>
-      <c r="B41" s="3" t="inlineStr">
+      <c r="B41" s="5" t="inlineStr">
         <is>
           <t>118.69.182.224:8879</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="C41" s="5" t="inlineStr"/>
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>Bien Hoa</t>
         </is>
       </c>
-      <c r="E41" s="3" t="inlineStr">
+      <c r="E41" s="5" t="inlineStr">
         <is>
           <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>http://123.25.63.30:8888</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B42" s="5" t="inlineStr">
         <is>
           <t>123.25.63.30:8888</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr"/>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="3" t="inlineStr">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>http://123.31.31.119:49163</t>
         </is>
       </c>
-      <c r="B43" s="3" t="inlineStr">
+      <c r="B43" s="5" t="inlineStr">
         <is>
           <t>123.31.31.119:49163</t>
         </is>
       </c>
-      <c r="C43" s="3" t="inlineStr">
+      <c r="C43" s="5" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
         <is>
           <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="3" t="inlineStr">
+      <c r="A44" s="4" t="inlineStr">
         <is>
           <t>http://123.31.31.125:49163</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
+      <c r="B44" s="5" t="inlineStr">
         <is>
           <t>123.31.31.125:49163</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C44" s="5" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
         <is>
           <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="4" t="inlineStr">
         <is>
           <t>http://123.31.36.63:8002</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B45" s="5" t="inlineStr">
         <is>
           <t>123.31.36.63:8002</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C45" s="5" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>http://14.241.253.96:8081</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
+      <c r="B46" s="5" t="inlineStr">
         <is>
           <t>14.241.253.96:8081</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr"/>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="E46" s="5" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>http://14.241.253.96:8082</t>
         </is>
       </c>
-      <c r="B47" s="3" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>14.241.253.96:8082</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
-      <c r="D47" s="3" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E47" s="3" t="inlineStr">
+      <c r="E47" s="5" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>http://160.191.101.129:9001</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>160.191.101.129:9001</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr"/>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
         <is>
           <t>Gplay Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>http://171.244.38.92:7001</t>
         </is>
       </c>
-      <c r="B49" s="3" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>171.244.38.92:7001</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D49" s="3" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E49" s="3" t="inlineStr">
+      <c r="E49" s="5" t="inlineStr">
         <is>
           <t>Viettel Group</t>
         </is>
@@ -1643,72 +1653,72 @@
           <t>http://183.91.187.108:8888</t>
         </is>
       </c>
-      <c r="B50" s="2" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
         <is>
           <t>183.91.187.108:8888</t>
         </is>
       </c>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr">
+      <c r="C50" s="3" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E50" s="2" t="inlineStr">
+      <c r="E50" s="3" t="inlineStr">
         <is>
           <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>http://210.211.98.79:8080</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B51" s="5" t="inlineStr">
         <is>
           <t>210.211.98.79:8080</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C51" s="5" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
         <is>
           <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="3" t="inlineStr">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>http://210.211.98.79:8081</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>210.211.98.79:8081</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
         <is>
           <t>Viettel - CHT Company Ltd</t>
         </is>
@@ -1720,122 +1730,122 @@
           <t>http://210.211.99.108:8080</t>
         </is>
       </c>
-      <c r="B53" s="2" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>210.211.99.108:8080</t>
         </is>
       </c>
-      <c r="C53" s="2" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
         <is>
           <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>http://42.116.12.202:9001</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
+      <c r="B54" s="5" t="inlineStr">
         <is>
           <t>42.116.12.202:9001</t>
         </is>
       </c>
-      <c r="C54" s="3" t="inlineStr"/>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="C54" s="5" t="inlineStr"/>
+      <c r="D54" s="5" t="inlineStr">
         <is>
           <t>Thu Dau Mot</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
+      <c r="E54" s="5" t="inlineStr">
         <is>
           <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>http://42.118.60.193:7001</t>
         </is>
       </c>
-      <c r="B55" s="3" t="inlineStr">
+      <c r="B55" s="5" t="inlineStr">
         <is>
           <t>42.118.60.193:7001</t>
         </is>
       </c>
-      <c r="C55" s="3" t="inlineStr">
+      <c r="C55" s="5" t="inlineStr">
         <is>
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
         <is>
           <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>http://49.213.88.170:7001</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" s="5" t="inlineStr">
         <is>
           <t>49.213.88.170:7001</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C56" s="5" t="inlineStr">
         <is>
           <t>10.3.6.0</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D56" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E56" s="5" t="inlineStr">
         <is>
           <t>VNG Corporation</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>https://103.238.209.174</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>103.238.209.174</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr"/>
-      <c r="D57" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E57" s="3" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr"/>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
         <is>
           <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
@@ -1847,18 +1857,18 @@
           <t>https://103.3.252.106:7002</t>
         </is>
       </c>
-      <c r="B58" s="2" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>103.3.252.106:7002</t>
         </is>
       </c>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr"/>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
         <is>
           <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
@@ -1870,45 +1880,45 @@
           <t>https://103.3.252.107:7002</t>
         </is>
       </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>103.3.252.107:7002</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr"/>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr"/>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
         <is>
           <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="3" t="inlineStr">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>https://103.82.192.168</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr">
+      <c r="B60" s="5" t="inlineStr">
         <is>
           <t>103.82.192.168</t>
         </is>
       </c>
-      <c r="C60" s="3" t="inlineStr">
+      <c r="C60" s="5" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D60" s="3" t="inlineStr">
+      <c r="D60" s="5" t="inlineStr">
         <is>
           <t>Da Nang</t>
         </is>
       </c>
-      <c r="E60" s="3" t="inlineStr">
+      <c r="E60" s="5" t="inlineStr">
         <is>
           <t>CLOUDFLY CORPORATION</t>
         </is>
@@ -1920,41 +1930,41 @@
           <t>https://118.69.32.193:3068</t>
         </is>
       </c>
-      <c r="B61" s="2" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>118.69.32.193:3068</t>
         </is>
       </c>
-      <c r="C61" s="2" t="inlineStr"/>
-      <c r="D61" s="2" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr"/>
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>Thu Dau Mot</t>
         </is>
       </c>
-      <c r="E61" s="2" t="inlineStr">
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="3" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>https://123.31.36.60</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr">
+      <c r="B62" s="5" t="inlineStr">
         <is>
           <t>123.31.36.60</t>
         </is>
       </c>
-      <c r="C62" s="3" t="inlineStr"/>
-      <c r="D62" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E62" s="3" t="inlineStr">
+      <c r="C62" s="5" t="inlineStr"/>
+      <c r="D62" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -1966,18 +1976,18 @@
           <t>https://14.238.93.114:9184</t>
         </is>
       </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="B63" s="3" t="inlineStr">
         <is>
           <t>14.238.93.114:9184</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr"/>
-      <c r="D63" s="2" t="inlineStr">
+      <c r="C63" s="3" t="inlineStr"/>
+      <c r="D63" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E63" s="2" t="inlineStr">
+      <c r="E63" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
@@ -1989,41 +1999,41 @@
           <t>https://14.238.93.114:9185</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>14.238.93.114:9185</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr"/>
-      <c r="D64" s="2" t="inlineStr">
+      <c r="C64" s="3" t="inlineStr"/>
+      <c r="D64" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E64" s="2" t="inlineStr">
+      <c r="E64" s="3" t="inlineStr">
         <is>
           <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="3" t="inlineStr">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>https://14.248.84.7</t>
         </is>
       </c>
-      <c r="B65" s="3" t="inlineStr">
+      <c r="B65" s="5" t="inlineStr">
         <is>
           <t>14.248.84.7</t>
         </is>
       </c>
-      <c r="C65" s="3" t="inlineStr"/>
-      <c r="D65" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E65" s="3" t="inlineStr">
+      <c r="C65" s="5" t="inlineStr"/>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
         <is>
           <t>Vietnam Posts and Telecommunications Group</t>
         </is>
@@ -2035,18 +2045,18 @@
           <t>https://183.91.187.108:8890</t>
         </is>
       </c>
-      <c r="B66" s="2" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>183.91.187.108:8890</t>
         </is>
       </c>
-      <c r="C66" s="2" t="inlineStr"/>
-      <c r="D66" s="2" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr"/>
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E66" s="2" t="inlineStr">
+      <c r="E66" s="3" t="inlineStr">
         <is>
           <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
         </is>
@@ -2058,41 +2068,41 @@
           <t>https://210.211.99.108</t>
         </is>
       </c>
-      <c r="B67" s="2" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>210.211.99.108</t>
         </is>
       </c>
-      <c r="C67" s="2" t="inlineStr"/>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr"/>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
         <is>
           <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>https://210.245.45.90</t>
         </is>
       </c>
-      <c r="B68" s="3" t="inlineStr">
+      <c r="B68" s="5" t="inlineStr">
         <is>
           <t>210.245.45.90</t>
         </is>
       </c>
-      <c r="C68" s="3" t="inlineStr"/>
-      <c r="D68" s="3" t="inlineStr">
+      <c r="C68" s="5" t="inlineStr"/>
+      <c r="D68" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E68" s="3" t="inlineStr">
+      <c r="E68" s="5" t="inlineStr">
         <is>
           <t>Dai IP cap cho Cong ty TNHH Nguon Viet Nam</t>
         </is>
@@ -2100,6 +2110,75 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:E68"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId67"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-10-08 15:05:43
</commit_message>
<xml_diff>
--- a/WebLogic-VN-confirmed.xlsx
+++ b/WebLogic-VN-confirmed.xlsx
@@ -713,35 +713,35 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>https://congbothongtin.ssc.gov.vn</t>
+          <t>https://app.pvfcco.com.vn</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.107</t>
+          <t>14.238.99.84</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Tan An</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>https://cskh.temxacthuc.vn:8081</t>
+          <t>https://congbothongtin.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19:8081</t>
+          <t>103.3.252.107</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr"/>
@@ -752,19 +752,19 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>https://dvctn.vst.mof.gov.vn</t>
+          <t>https://cskh.temxacthuc.vn:8081</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.41</t>
+          <t>123.30.208.19:8081</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
@@ -775,19 +775,19 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>https://epayment.customs.gov.vn</t>
+          <t>https://dvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>103.248.160.36</t>
+          <t>45.120.230.40</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
@@ -798,138 +798,134 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Customs Statistics</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>https://hrs.mfmldb.com.vn:8184</t>
+          <t>https://dvctn.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>14.238.93.114:8184</t>
+          <t>45.120.230.41</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>https://hrs.mfmldb.com.vn:8185</t>
+          <t>https://epayment.customs.gov.vn</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>14.238.93.114:8185</t>
+          <t>103.248.160.36</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr"/>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Department of Information Technology and Customs Statistics</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>https://ids.ssc.gov.vn</t>
+          <t>https://esign.pvfcco.com.vn</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.106</t>
+          <t>14.238.99.83</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Tan An</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>https://kimdental.vn</t>
+          <t>https://hrs.mfmldb.com.vn:8184</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>42.115.41.28</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>12.2.1.3.0</t>
-        </is>
-      </c>
+          <t>14.238.93.114:8184</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr"/>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>https://mail.dailybanxetai.com</t>
+          <t>https://hrs.mfmldb.com.vn:8185</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19</t>
+          <t>14.238.93.114:8185</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>https://mail.dailybanxetai.com:8098</t>
+          <t>https://ids.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19:8098</t>
+          <t>103.3.252.106</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr"/>
@@ -940,19 +936,19 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.vn</t>
+          <t>https://mail.dailybanxetai.com</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.40</t>
+          <t>123.30.208.19</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -963,19 +959,19 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>https://mof.gov.vn</t>
+          <t>https://mail.dailybanxetai.com:8098</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.51</t>
+          <t>123.30.208.19:8098</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr"/>
@@ -986,19 +982,19 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>https://mps.gov.vn</t>
+          <t>https://mla.toaan.gov.vn</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>42.1.75.65</t>
+          <t>123.30.24.180</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1009,76 +1005,80 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Mobifone Corporation</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>https://pritos.cloud:3068</t>
+          <t>https://orabi.kimdental.vn</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>115.75.20.142:3068</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr"/>
+          <t>42.115.41.28</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>12.2.1.3.0</t>
+        </is>
+      </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Thi Tran Long Dien</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>https://pvfcco.com.vn</t>
+          <t>https://pritos.cloud:3068</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>14.238.99.83</t>
+          <t>115.75.20.142:3068</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Tan An</t>
+          <t>Thi Tran Long Dien</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>https://pvfcco.com.vn</t>
+          <t>https://rsaweb.mps.gov.vn</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>14.238.99.84</t>
+          <t>42.1.75.65</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Tan An</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Mobifone Corporation</t>
         </is>
       </c>
     </row>
@@ -1108,12 +1108,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>https://toaan.gov.vn</t>
+          <t>https://tracuudvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>123.30.24.180</t>
+          <t>45.120.230.51</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr"/>
@@ -1124,14 +1124,14 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>https://vinpro.net</t>
+          <t>https://www.vinpro.net</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -1154,7 +1154,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>https://xsmb360.com</t>
+          <t>https://www.xsmb360.com</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">

</xml_diff>

<commit_message>
vault backup: 2026-10-08 16:36:24
</commit_message>
<xml_diff>
--- a/WebLogic-VN-confirmed.xlsx
+++ b/WebLogic-VN-confirmed.xlsx
@@ -10,7 +10,7 @@
     <sheet name="WebLogic VN" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WebLogic VN'!$A$1:$E$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'WebLogic VN'!$A$1:$E$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -621,58 +621,58 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>http://gasdaiminhquang.direct.quickconnect.to:82</t>
+          <t>http://apvs1.dlp.com.tw:9001</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>14.241.227.70:82</t>
+          <t>113.160.129.228:9001</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr"/>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>http://hddt.agimexpharm.com:8081</t>
+          <t>http://apvs1.dlp.com.tw:9002</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>113.161.212.113:8081</t>
+          <t>113.160.129.228:9002</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Long Xuyen</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>http://mail.xboss.vn:9999</t>
+          <t>http://gasdaiminhquang.direct.quickconnect.to:82</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>103.104.121.208:9999</t>
+          <t>14.241.227.70:82</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr"/>
@@ -683,65 +683,65 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Viet Storage Technology Joint Stock Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>http://sso.vietinbank.vn</t>
+          <t>http://hddt.agimexpharm.com:8081</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>203.189.29.33</t>
+          <t>113.161.212.113:8081</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Long Xuyen</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>VIETNAM Joint Stock Commercial Bank for Industry and Trade</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>https://app.pvfcco.com.vn</t>
+          <t>http://mail.xboss.vn:9999</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>14.238.99.84</t>
+          <t>103.104.121.208:9999</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr"/>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Tan An</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>https://congbothongtin.ssc.gov.vn</t>
+          <t>http://sso.vietinbank.vn</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.107</t>
+          <t>203.189.29.33</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr"/>
@@ -752,111 +752,111 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>VIETNAM Joint Stock Commercial Bank for Industry and Trade</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>https://cskh.temxacthuc.vn:8081</t>
+          <t>http://thongbaotenmien.vn</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19:8081</t>
+          <t>203.119.73.12:80</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr"/>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Vietnam Internet network information center (VNNIC)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>https://dvc.vst.mof.gov.vn</t>
+          <t>http://www.dtsweb.tech:8081</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.40</t>
+          <t>113.161.81.238:8081</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr"/>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>https://dvctn.vst.mof.gov.vn</t>
+          <t>http://www.dtsweb.tech:9001</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.41</t>
+          <t>113.161.81.238:9001</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr"/>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>https://epayment.customs.gov.vn</t>
+          <t>http://www.hddt.agimexpharm.com:8082</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>103.248.160.36</t>
+          <t>113.161.212.113:8082</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr"/>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Long Xuyen</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Department of Information Technology and Customs Statistics</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>https://esign.pvfcco.com.vn</t>
+          <t>https://app.pvfcco.com.vn</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>14.238.99.83</t>
+          <t>14.238.99.84</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr"/>
@@ -874,58 +874,58 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>https://hrs.mfmldb.com.vn:8184</t>
+          <t>https://congbothongtin.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>14.238.93.114:8184</t>
+          <t>103.3.252.107</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr"/>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>https://hrs.mfmldb.com.vn:8185</t>
+          <t>https://cskh.temxacthuc.vn</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>14.238.93.114:8185</t>
+          <t>123.30.208.19</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr"/>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>VNPT Corp</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>https://ids.ssc.gov.vn</t>
+          <t>https://cskh.temxacthuc.vn:8081</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.106</t>
+          <t>123.30.208.19:8081</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr"/>
@@ -936,19 +936,19 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>https://mail.dailybanxetai.com</t>
+          <t>https://dvc.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19</t>
+          <t>45.120.230.40</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr"/>
@@ -959,19 +959,19 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>https://mail.dailybanxetai.com:8098</t>
+          <t>https://dvctn.vst.mof.gov.vn</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>123.30.208.19:8098</t>
+          <t>45.120.230.41</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr"/>
@@ -982,19 +982,19 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>https://mla.toaan.gov.vn</t>
+          <t>https://epayment.customs.gov.vn</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>123.30.24.180</t>
+          <t>103.248.160.36</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr"/>
@@ -1005,115 +1005,111 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Department of Information Technology and Customs Statistics</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>https://orabi.kimdental.vn</t>
+          <t>https://esign.pvfcco.com.vn</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>42.115.41.28</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>12.2.1.3.0</t>
-        </is>
-      </c>
+          <t>14.238.99.83</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr"/>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Tan An</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>https://pritos.cloud:3068</t>
+          <t>https://hrs.mfmldb.com.vn:8184</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>115.75.20.142:3068</t>
+          <t>14.238.93.114:8184</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr"/>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Thi Tran Long Dien</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>https://rsaweb.mps.gov.vn</t>
+          <t>https://hrs.mfmldb.com.vn:8185</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>42.1.75.65</t>
+          <t>14.238.93.114:8185</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr"/>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Mobifone Corporation</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>https://thongbaotenmien.vn</t>
+          <t>https://ids.ssc.gov.vn</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>203.119.73.12</t>
+          <t>103.3.252.106</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr"/>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Vietnam Internet network information center (VNNIC)</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>https://tracuudvc.vst.mof.gov.vn</t>
+          <t>https://mail.dailybanxetai.com:8098</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>45.120.230.51</t>
+          <t>123.30.208.19:8098</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr"/>
@@ -1124,19 +1120,19 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Creative Communication Vietnam Joint Stock Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>https://www.vinpro.net</t>
+          <t>https://mla.toaan.gov.vn</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>103.238.209.204</t>
+          <t>123.30.24.180</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr"/>
@@ -1147,265 +1143,257 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>https://orabi.kimdental.vn</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>42.115.41.28</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>12.2.1.3.0</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>https://pritos.cloud:3068</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>115.75.20.142:3068</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Thi Tran Long Dien</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Viettel Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>https://rsaweb.mps.gov.vn</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>42.1.75.65</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Mobifone Corporation</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>https://thongbaotenmien.vn</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>203.119.73.12</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Vietnam Internet network information center (VNNIC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>https://tracuudvc.vst.mof.gov.vn</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>45.120.230.51</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Creative Communication Vietnam Joint Stock Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>https://www.vinpro.net</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>103.238.209.204</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
           <t>https://www.xsmb360.com</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>103.82.194.3</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>14.1.1.0.0</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>Tra Vinh</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>CLOUDFLY CORPORATION</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>http://103.104.121.206:9999</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>103.104.121.206:9999</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr"/>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Viet Storage Technology Joint Stock Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>http://103.104.121.207:9999</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>103.104.121.207:9999</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="inlineStr"/>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="E32" s="5" t="inlineStr">
-        <is>
-          <t>Viet Storage Technology Joint Stock Company</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>http://113.160.129.149:8888</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>113.160.129.149:8888</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr"/>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>Hai Duong</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
-        <is>
-          <t>http://113.160.201.159:7001</t>
-        </is>
-      </c>
-      <c r="B34" s="5" t="inlineStr">
-        <is>
-          <t>113.160.201.159:7001</t>
-        </is>
-      </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Thai Binh</t>
-        </is>
-      </c>
-      <c r="E34" s="5" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>http://113.161.43.248:9001</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>113.161.43.248:9001</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr"/>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t>http://113.163.187.3:27001</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>113.163.187.3:27001</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>Phan Rang-Thap Cham</t>
-        </is>
-      </c>
-      <c r="E36" s="5" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>http://113.185.0.60:8080</t>
+          <t>http://103.104.121.206:9999</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>113.185.0.60:8080</t>
+          <t>103.104.121.206:9999</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr"/>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>http://113.185.19.167:8080</t>
+          <t>http://103.104.121.207:9999</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>113.185.19.167:8080</t>
+          <t>103.104.121.207:9999</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr"/>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viet Storage Technology Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>http://117.4.241.247:1112</t>
+          <t>http://113.160.129.149:8888</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>117.4.241.247:1112</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
+          <t>113.160.129.149:8888</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr"/>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Hai Duong</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>http://117.4.32.40:1111</t>
+          <t>http://113.160.201.159:7001</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>117.4.32.40:1111</t>
+          <t>113.160.201.159:7001</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -1415,53 +1403,57 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Thai Binh</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>http://118.69.182.224:8879</t>
+          <t>http://113.161.43.248:9001</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>118.69.182.224:8879</t>
+          <t>113.161.43.248:9001</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr"/>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Bien Hoa</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>http://123.25.63.30:8888</t>
+          <t>http://113.163.187.3:27001</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>123.25.63.30:8888</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr"/>
+          <t>113.163.187.3:27001</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Phan Rang-Thap Cham</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -1473,19 +1465,15 @@
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>http://123.31.31.119:49163</t>
+          <t>http://113.185.0.60:8080</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>123.31.31.119:49163</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
+          <t>113.185.0.60:8080</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr"/>
       <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -1493,26 +1481,22 @@
       </c>
       <c r="E43" s="5" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>http://123.31.31.125:49163</t>
+          <t>http://113.185.19.167:8080</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>123.31.31.125:49163</t>
-        </is>
-      </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
+          <t>113.185.19.167:8080</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr"/>
       <c r="D44" s="5" t="inlineStr">
         <is>
           <t>Hanoi</t>
@@ -1520,24 +1504,24 @@
       </c>
       <c r="E44" s="5" t="inlineStr">
         <is>
-          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>http://123.31.36.63:8002</t>
+          <t>http://117.4.241.247:1112</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>123.31.36.63:8002</t>
+          <t>117.4.241.247:1112</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>14.1.1.0.0</t>
+          <t>10.3.6.0</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
@@ -1547,138 +1531,142 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>http://14.241.253.96:8081</t>
+          <t>http://117.4.32.40:1111</t>
         </is>
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>14.241.253.96:8081</t>
-        </is>
-      </c>
-      <c r="C46" s="5" t="inlineStr"/>
+          <t>117.4.32.40:1111</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>http://14.241.253.96:8082</t>
+          <t>http://118.69.182.224:8879</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>14.241.253.96:8082</t>
+          <t>118.69.182.224:8879</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr"/>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Bien Hoa</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>http://160.191.101.129:9001</t>
+          <t>http://118.69.182.224:9079</t>
         </is>
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>160.191.101.129:9001</t>
+          <t>118.69.182.224:9079</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr"/>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Bien Hoa</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Gplay Joint Stock Company</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>http://171.244.38.92:7001</t>
+          <t>http://123.25.63.30:8888</t>
         </is>
       </c>
       <c r="B49" s="5" t="inlineStr">
         <is>
-          <t>171.244.38.92:7001</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
+          <t>123.25.63.30:8888</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr"/>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>Viettel Group</t>
+          <t>VNPT Corp</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>http://183.91.187.108:8888</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>183.91.187.108:8888</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr"/>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>http://123.31.31.119:49163</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>123.31.31.119:49163</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>http://210.211.98.79:8080</t>
+          <t>http://123.31.31.125:49163</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr">
         <is>
-          <t>210.211.98.79:8080</t>
+          <t>123.31.31.125:49163</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
@@ -1693,19 +1681,19 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Viettel - CHT Company Ltd</t>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>http://210.211.98.79:8081</t>
+          <t>http://123.31.36.63:8002</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr">
         <is>
-          <t>210.211.98.79:8081</t>
+          <t>123.31.36.63:8002</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
@@ -1720,192 +1708,188 @@
       </c>
       <c r="E52" s="5" t="inlineStr">
         <is>
-          <t>Viettel - CHT Company Ltd</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>http://210.211.99.108:8080</t>
-        </is>
-      </c>
-      <c r="B53" s="3" t="inlineStr">
-        <is>
-          <t>210.211.99.108:8080</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>14.1.1.0.0</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>Viettel - CHT Company Ltd</t>
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>http://14.225.11.33:9001</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>14.225.11.33:9001</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>VIETNAM POSTS AND TELECOMMUNICATIONS GROUP</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>http://42.116.12.202:9001</t>
+          <t>http://14.241.253.96:8081</t>
         </is>
       </c>
       <c r="B54" s="5" t="inlineStr">
         <is>
-          <t>42.116.12.202:9001</t>
+          <t>14.241.253.96:8081</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr"/>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Thu Dau Mot</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>http://42.118.60.193:7001</t>
+          <t>http://14.241.253.96:8082</t>
         </is>
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>42.118.60.193:7001</t>
-        </is>
-      </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
+          <t>14.241.253.96:8082</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr"/>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Vietnam Posts and Telecommunications Group</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>http://49.213.88.170:7001</t>
+          <t>http://160.191.101.129:9001</t>
         </is>
       </c>
       <c r="B56" s="5" t="inlineStr">
         <is>
-          <t>49.213.88.170:7001</t>
-        </is>
-      </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>10.3.6.0</t>
-        </is>
-      </c>
+          <t>160.191.101.129:9001</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr"/>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
         <is>
-          <t>VNG Corporation</t>
+          <t>Gplay Joint Stock Company</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>https://103.238.209.174</t>
+          <t>http://171.244.38.92:7001</t>
         </is>
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>103.238.209.174</t>
-        </is>
-      </c>
-      <c r="C57" s="5" t="inlineStr"/>
+          <t>171.244.38.92:7001</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>VINGROUP JOINT STOCK COMPANY</t>
+          <t>Viettel Group</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>https://103.3.252.106:7002</t>
+          <t>http://183.91.187.108:8888</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>103.3.252.106:7002</t>
+          <t>183.91.187.108:8888</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr"/>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Ho Chi Minh City</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+          <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>https://103.3.252.107:7002</t>
-        </is>
-      </c>
-      <c r="B59" s="3" t="inlineStr">
-        <is>
-          <t>103.3.252.107:7002</t>
-        </is>
-      </c>
-      <c r="C59" s="3" t="inlineStr"/>
-      <c r="D59" s="3" t="inlineStr">
-        <is>
-          <t>Hanoi</t>
-        </is>
-      </c>
-      <c r="E59" s="3" t="inlineStr">
-        <is>
-          <t>Cong ty CP Truyen thong quoc te Incom</t>
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>http://210.211.98.79:8080</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>210.211.98.79:8080</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>https://103.82.192.168</t>
+          <t>http://210.211.98.79:8081</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr">
         <is>
-          <t>103.82.192.168</t>
+          <t>210.211.98.79:8081</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
@@ -1915,116 +1899,128 @@
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Da Nang</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
         <is>
-          <t>CLOUDFLY CORPORATION</t>
+          <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>https://118.69.32.193:3068</t>
+          <t>http://210.211.99.108:8080</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>118.69.32.193:3068</t>
-        </is>
-      </c>
-      <c r="C61" s="3" t="inlineStr"/>
+          <t>210.211.99.108:8080</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Thu Dau Mot</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>FPT Telecom Company</t>
+          <t>Viettel - CHT Company Ltd</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>https://123.31.36.60</t>
+          <t>http://42.116.12.202:9001</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr">
         <is>
-          <t>123.31.36.60</t>
+          <t>42.116.12.202:9001</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr"/>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Hanoi</t>
+          <t>Thu Dau Mot</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>FPT Telecom Company</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>https://14.238.93.114:9184</t>
-        </is>
-      </c>
-      <c r="B63" s="3" t="inlineStr">
-        <is>
-          <t>14.238.93.114:9184</t>
-        </is>
-      </c>
-      <c r="C63" s="3" t="inlineStr"/>
-      <c r="D63" s="3" t="inlineStr">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>http://42.118.60.193:7001</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>42.118.60.193:7001</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>http://49.213.88.170:7001</t>
+        </is>
+      </c>
+      <c r="B64" s="5" t="inlineStr">
+        <is>
+          <t>49.213.88.170:7001</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>10.3.6.0</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E63" s="3" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>https://14.238.93.114:9185</t>
-        </is>
-      </c>
-      <c r="B64" s="3" t="inlineStr">
-        <is>
-          <t>14.238.93.114:9185</t>
-        </is>
-      </c>
-      <c r="C64" s="3" t="inlineStr"/>
-      <c r="D64" s="3" t="inlineStr">
-        <is>
-          <t>Ho Chi Minh City</t>
-        </is>
-      </c>
-      <c r="E64" s="3" t="inlineStr">
-        <is>
-          <t>VNPT Corp</t>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>VNG Corporation</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>https://14.248.84.7</t>
+          <t>https://103.238.209.174</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>14.248.84.7</t>
+          <t>103.238.209.174</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr"/>
@@ -2035,42 +2031,42 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Vietnam Posts and Telecommunications Group</t>
+          <t>VINGROUP JOINT STOCK COMPANY</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>https://183.91.187.108:8890</t>
+          <t>https://103.3.252.106:7002</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>183.91.187.108:8890</t>
+          <t>103.3.252.106:7002</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr"/>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Ho Chi Minh City</t>
+          <t>Hanoi</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>https://210.211.99.108</t>
+          <t>https://103.3.252.107:7002</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>210.211.99.108</t>
+          <t>103.3.252.107:7002</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr"/>
@@ -2081,35 +2077,223 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Viettel - CHT Company Ltd</t>
+          <t>Cong ty CP Truyen thong quoc te Incom</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
+          <t>https://103.82.192.168</t>
+        </is>
+      </c>
+      <c r="B68" s="5" t="inlineStr">
+        <is>
+          <t>103.82.192.168</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>14.1.1.0.0</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>Da Nang</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr">
+        <is>
+          <t>CLOUDFLY CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>https://118.69.32.193:3068</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>118.69.32.193:3068</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr"/>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>Thu Dau Mot</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>FPT Telecom Company</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>https://123.31.36.60</t>
+        </is>
+      </c>
+      <c r="B70" s="5" t="inlineStr">
+        <is>
+          <t>123.31.36.60</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr"/>
+      <c r="D70" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>https://14.238.93.114:9184</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>14.238.93.114:9184</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr"/>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>https://14.238.93.114:9185</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>14.238.93.114:9185</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr"/>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>VNPT Corp</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>https://14.248.84.7</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>14.248.84.7</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr"/>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Vietnam Posts and Telecommunications Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>https://183.91.187.108:8890</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>183.91.187.108:8890</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Ho Chi Minh City</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>GLOBAL TECHNOLOGY - TELECOMMUNICATIONS CORPORATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>https://210.211.99.108</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>210.211.99.108</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr"/>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Hanoi</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Viettel - CHT Company Ltd</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
           <t>https://210.245.45.90</t>
         </is>
       </c>
-      <c r="B68" s="5" t="inlineStr">
+      <c r="B76" s="5" t="inlineStr">
         <is>
           <t>210.245.45.90</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr"/>
-      <c r="D68" s="5" t="inlineStr">
+      <c r="C76" s="5" t="inlineStr"/>
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>Ho Chi Minh City</t>
         </is>
       </c>
-      <c r="E68" s="5" t="inlineStr">
+      <c r="E76" s="5" t="inlineStr">
         <is>
           <t>Dai IP cap cho Cong ty TNHH Nguon Viet Nam</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E68"/>
+  <autoFilter ref="A1:E76"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
@@ -2178,6 +2362,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId65"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId66"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A76" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>